<commit_message>
docs(order-history): format 13.3 Open Questions sheet (header/wrap/verdict color-code)
</commit_message>
<xml_diff>
--- a/order_history/13.3-order-details-page/13.3 - Order Details Page.xlsx
+++ b/order_history/13.3-order-details-page/13.3 - Order Details Page.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -53,8 +53,15 @@
       <color rgb="FF0563C1"/>
       <u val="single"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -103,6 +110,26 @@
         <bgColor rgb="FFBFBFBF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8CBAD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFE699"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDEBF7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border/>
@@ -124,7 +151,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -179,6 +206,21 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5549,431 +5591,431 @@
   <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col width="9" customWidth="1" style="19" min="1" max="1"/>
-    <col width="32" customWidth="1" style="19" min="2" max="2"/>
-    <col width="18" customWidth="1" style="19" min="3" max="3"/>
-    <col width="55" customWidth="1" style="19" min="4" max="4"/>
-    <col width="55" customWidth="1" style="19" min="5" max="26"/>
-    <col width="28" customWidth="1" style="19" min="6" max="6"/>
-    <col width="34" customWidth="1" style="19" min="7" max="7"/>
-    <col width="60" customWidth="1" style="19" min="8" max="8"/>
+    <col width="8" customWidth="1" style="19" min="1" max="1"/>
+    <col width="26" customWidth="1" style="19" min="2" max="2"/>
+    <col width="15" customWidth="1" style="19" min="3" max="3"/>
+    <col width="46" customWidth="1" style="19" min="4" max="4"/>
+    <col width="50" customWidth="1" style="19" min="5" max="26"/>
+    <col width="24" customWidth="1" style="19" min="6" max="6"/>
+    <col width="30" customWidth="1" style="19" min="7" max="7"/>
+    <col width="52" customWidth="1" style="19" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="0" t="inlineStr">
+    <row r="1" ht="30" customHeight="1" s="19">
+      <c r="A1" s="20" t="inlineStr">
         <is>
           <t>Req</t>
         </is>
       </c>
-      <c r="B1" s="0" t="inlineStr">
+      <c r="B1" s="20" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="C1" s="0" t="inlineStr">
+      <c r="C1" s="20" t="inlineStr">
         <is>
           <t>Verdict</t>
         </is>
       </c>
-      <c r="D1" s="0" t="inlineStr">
+      <c r="D1" s="20" t="inlineStr">
         <is>
           <t>Open Question / What is needed</t>
         </is>
       </c>
-      <c r="E1" s="0" t="inlineStr">
+      <c r="E1" s="20" t="inlineStr">
         <is>
           <t>Dependency (blocking story + Jira)</t>
         </is>
       </c>
-      <c r="F1" s="0" t="inlineStr">
+      <c r="F1" s="20" t="inlineStr">
         <is>
           <t>Assignee</t>
         </is>
       </c>
-      <c r="G1" s="0" t="inlineStr">
+      <c r="G1" s="20" t="inlineStr">
         <is>
           <t>Sprint / Jira status</t>
         </is>
       </c>
-      <c r="H1" s="0" t="inlineStr">
+      <c r="H1" s="20" t="inlineStr">
         <is>
           <t>Decision / Current direction</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="0" t="inlineStr">
+      <c r="A2" s="21" t="inlineStr">
         <is>
           <t>13.3-c</t>
         </is>
       </c>
-      <c r="B2" s="0" t="inlineStr">
+      <c r="B2" s="21" t="inlineStr">
         <is>
           <t>Booth Number</t>
         </is>
       </c>
-      <c r="C2" s="0" t="inlineStr">
+      <c r="C2" s="22" t="inlineStr">
         <is>
           <t>Not Deliverable</t>
         </is>
       </c>
-      <c r="D2" s="0" t="inlineStr">
+      <c r="D2" s="21" t="inlineStr">
         <is>
           <t>Is a physical stall/booth number required on the details page? If yes, from where (it is assigned externally after purchase)?</t>
         </is>
       </c>
-      <c r="E2" s="0" t="inlineStr">
+      <c r="E2" s="21" t="inlineStr">
         <is>
           <t>No producing story. Lead only: 'Booth Sign Print Page' (Confluence: SBE - Admin Panel Page 2) references company+show 'assigned booth numbers' (not order-linked).</t>
         </is>
       </c>
-      <c r="F2" s="0" t="inlineStr">
+      <c r="F2" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G2" s="0" t="inlineStr">
+      <c r="G2" s="21" t="inlineStr">
         <is>
           <t>— (no story / parked)</t>
         </is>
       </c>
-      <c r="H2" s="0" t="inlineStr">
+      <c r="H2" s="21" t="inlineStr">
         <is>
           <t>PARKED. No order-linked booth-number source exists (notification-template.seeder.ts:668 = assigned externally, separate notification). Awaiting team direction.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="0" t="inlineStr">
+      <c r="A3" s="21" t="inlineStr">
         <is>
           <t>13.3-f</t>
         </is>
       </c>
-      <c r="B3" s="0" t="inlineStr">
+      <c r="B3" s="21" t="inlineStr">
         <is>
           <t>Booth Type (Standard/Premium/Corner)</t>
         </is>
       </c>
-      <c r="C3" s="0" t="inlineStr">
+      <c r="C3" s="22" t="inlineStr">
         <is>
           <t>Not Deliverable</t>
         </is>
       </c>
-      <c r="D3" s="0" t="inlineStr">
+      <c r="D3" s="21" t="inlineStr">
         <is>
           <t>Is Booth Type actually required here, or was it added arbitrarily by the BA?</t>
         </is>
       </c>
-      <c r="E3" s="0" t="inlineStr">
+      <c r="E3" s="21" t="inlineStr">
         <is>
           <t>No story located. Classification data does not exist (ProductType = product family only; purchased-booths 'boothType' is derived size).</t>
         </is>
       </c>
-      <c r="F3" s="0" t="inlineStr">
+      <c r="F3" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G3" s="0" t="inlineStr">
+      <c r="G3" s="21" t="inlineStr">
         <is>
           <t>— (no story / parked)</t>
         </is>
       </c>
-      <c r="H3" s="0" t="inlineStr">
+      <c r="H3" s="21" t="inlineStr">
         <is>
           <t>PARKED. Not deliverable on current data; needs an upstream classification if genuinely required.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="0" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>13.3-g</t>
         </is>
       </c>
-      <c r="B4" s="0" t="inlineStr">
+      <c r="B4" s="21" t="inlineStr">
         <is>
           <t>Booth Upgrade ('Upgrade details, if any')</t>
         </is>
       </c>
-      <c r="C4" s="0" t="inlineStr">
+      <c r="C4" s="23" t="inlineStr">
         <is>
           <t>Blocked</t>
         </is>
       </c>
-      <c r="D4" s="0" t="inlineStr">
+      <c r="D4" s="21" t="inlineStr">
         <is>
           <t>Is 'Upgrade details' required on this page, and what would it show (upgrades are fresh purchases)?</t>
         </is>
       </c>
-      <c r="E4" s="0" t="inlineStr">
+      <c r="E4" s="21" t="inlineStr">
         <is>
           <t>'Booth Upgrade' user story — Confluence: SBE - Exhibitor Store Application (search 'Booth Upgrade' / 'Upgrade Booth'). No discrete Jira key found.</t>
         </is>
       </c>
-      <c r="F4" s="0" t="inlineStr">
+      <c r="F4" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G4" s="0" t="inlineStr">
+      <c r="G4" s="21" t="inlineStr">
         <is>
           <t>— (no sprint found)</t>
         </is>
       </c>
-      <c r="H4" s="0" t="inlineStr">
+      <c r="H4" s="21" t="inlineStr">
         <is>
           <t>BLOCKED on the Booth Upgrade story. No 'upgrade detail' is stored on the original order today.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="0" t="inlineStr">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>13.3-l</t>
         </is>
       </c>
-      <c r="B5" s="0" t="inlineStr">
+      <c r="B5" s="21" t="inlineStr">
         <is>
           <t>Gift Certificate line</t>
         </is>
       </c>
-      <c r="C5" s="0" t="inlineStr">
+      <c r="C5" s="23" t="inlineStr">
         <is>
           <t>Blocked</t>
         </is>
       </c>
-      <c r="D5" s="0" t="inlineStr">
+      <c r="D5" s="21" t="inlineStr">
         <is>
           <t>Awaiting a producer that redeems a gift certificate against an order (writes GiftCertificateRedeem).</t>
         </is>
       </c>
-      <c r="E5" s="0" t="inlineStr">
+      <c r="E5" s="21" t="inlineStr">
         <is>
           <t>Story 12.4 'Gift Cart Redemption' (Confluence: SBE - Exhibitor Store Application); Jira SBE-1069 'Gift Certificate Purchase and Redemption' (Epic).</t>
         </is>
       </c>
-      <c r="F5" s="0" t="inlineStr">
+      <c r="F5" s="21" t="inlineStr">
         <is>
           <t>Unassigned</t>
         </is>
       </c>
-      <c r="G5" s="0" t="inlineStr">
+      <c r="G5" s="21" t="inlineStr">
         <is>
           <t>To Do — backlog (no sprint)</t>
         </is>
       </c>
-      <c r="H5" s="0" t="inlineStr">
+      <c r="H5" s="21" t="inlineStr">
         <is>
           <t>BLOCKED. Omit the line via conditional display until SBE-1069 / Story 12.4 ships the redemption write-path.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="0" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>13.3-s</t>
         </is>
       </c>
-      <c r="B6" s="0" t="inlineStr">
+      <c r="B6" s="21" t="inlineStr">
         <is>
           <t>Download Invoice PDF</t>
         </is>
       </c>
-      <c r="C6" s="0" t="inlineStr">
+      <c r="C6" s="24" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
       </c>
-      <c r="D6" s="0" t="inlineStr">
+      <c r="D6" s="21" t="inlineStr">
         <is>
           <t>DECISION: invoice semantics A vs B — A = generate an order-level PDF from Order+OrderItems (any order, incl. unpaid); B = serve only persisted Invoice rows (paid orders only).</t>
         </is>
       </c>
-      <c r="E6" s="0" t="inlineStr">
+      <c r="E6" s="21" t="inlineStr">
         <is>
           <t>None — a team decision (inherited from 13.2's invoice deferral). pdfkit renderer exists but is subscription/Invoice-shaped.</t>
         </is>
       </c>
-      <c r="F6" s="0" t="inlineStr">
+      <c r="F6" s="21" t="inlineStr">
         <is>
           <t>13.3 team</t>
         </is>
       </c>
-      <c r="G6" s="0" t="inlineStr">
+      <c r="G6" s="21" t="inlineStr">
         <is>
           <t>Deferred — decision pending</t>
         </is>
       </c>
-      <c r="H6" s="0" t="inlineStr">
+      <c r="H6" s="21" t="inlineStr">
         <is>
           <t>DEFERRED pending the A-vs-B decision. Resolving it moves 13.3-s (and 13.3-ac invoice half) into build scope.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="0" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>13.3-t</t>
         </is>
       </c>
-      <c r="B7" s="0" t="inlineStr">
+      <c r="B7" s="21" t="inlineStr">
         <is>
           <t>Payment Schedule (salesperson-set)</t>
         </is>
       </c>
-      <c r="C7" s="0" t="inlineStr">
+      <c r="C7" s="23" t="inlineStr">
         <is>
           <t>Blocked</t>
         </is>
       </c>
-      <c r="D7" s="0" t="inlineStr">
+      <c r="D7" s="21" t="inlineStr">
         <is>
           <t>Salesperson payment plan must be written, LINKED TO THE ORDER, and surfaced to the exhibitor (today CartPaymentScheduleEntry is cart-only, no Order FK).</t>
         </is>
       </c>
-      <c r="E7" s="0" t="inlineStr">
+      <c r="E7" s="21" t="inlineStr">
         <is>
           <t>Visibility: SBE-1154 'Payment Schedule Visibility'. Producers: SBE-1109 'Shared Cart Payment Plan', SBE-1111 'Payment Schedule Management', SBE-1112 'Payment Plan Date Validation' -&gt; OM 24.8. (SBE-1132 'Payment Plan Management' -&gt; 24.8.)</t>
         </is>
       </c>
-      <c r="F7" s="0" t="inlineStr">
+      <c r="F7" s="21" t="inlineStr">
         <is>
           <t>SBE-1154: Prantik Saha; SBE-1109/1111/1112: Suman Paul</t>
         </is>
       </c>
-      <c r="G7" s="0" t="inlineStr">
+      <c r="G7" s="21" t="inlineStr">
         <is>
           <t>SBE-1154: To Do, backlog. SBE-1109/1111/1112: In Progress, SBE Sprint 5 (15 Jun-2 Jul).</t>
         </is>
       </c>
-      <c r="H7" s="0" t="inlineStr">
+      <c r="H7" s="21" t="inlineStr">
         <is>
           <t>BLOCKED on SBE-1154 (+ producers). Option (b): the /payments/checkout split flow already writes a per-installment schedule in PaymentTransaction - deliverable now if the team wants it.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="0" t="inlineStr">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>13.3-v</t>
         </is>
       </c>
-      <c r="B8" s="0" t="inlineStr">
+      <c r="B8" s="21" t="inlineStr">
         <is>
           <t>Download signed agreement</t>
         </is>
       </c>
-      <c r="C8" s="0" t="inlineStr">
+      <c r="C8" s="23" t="inlineStr">
         <is>
           <t>Blocked</t>
         </is>
       </c>
-      <c r="D8" s="0" t="inlineStr">
+      <c r="D8" s="21" t="inlineStr">
         <is>
           <t>Confirm the EXISTING composed-DOCX download endpoint (GET /agreement/signed/:orderId/download) is complete/final; is DOCX acceptable (vs PDF)? Is SBE-1158 superseded by it?</t>
         </is>
       </c>
-      <c r="E8" s="0" t="inlineStr">
+      <c r="E8" s="21" t="inlineStr">
         <is>
           <t>Code authored by Kshitiz under SBE-862 'Exhibitor Agreement &amp; Checkout Review' + SBE-869 'Signed Agreement Storage'. Separate story SBE-1158 'Download Agreement Option'.</t>
         </is>
       </c>
-      <c r="F8" s="0" t="inlineStr">
+      <c r="F8" s="21" t="inlineStr">
         <is>
           <t>SBE-862/869: Kshitiz; SBE-1158: Prantik Saha</t>
         </is>
       </c>
-      <c r="G8" s="0" t="inlineStr">
+      <c r="G8" s="21" t="inlineStr">
         <is>
           <t>SBE-862/869: In Progress, SBE Sprint 5. SBE-1158: To Do, backlog.</t>
         </is>
       </c>
-      <c r="H8" s="0" t="inlineStr">
+      <c r="H8" s="21" t="inlineStr">
         <is>
           <t>BLOCKED pending team confirmation of completion (SBE-862/869 in-flight) + reconciliation of SBE-1158 (possibly superseded). Reuse the existing endpoint; DOCX not PDF.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="0" t="inlineStr">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t>13.3-w</t>
         </is>
       </c>
-      <c r="B9" s="0" t="inlineStr">
+      <c r="B9" s="21" t="inlineStr">
         <is>
           <t>Onsite Contact information</t>
         </is>
       </c>
-      <c r="C9" s="0" t="inlineStr">
+      <c r="C9" s="23" t="inlineStr">
         <is>
           <t>Blocked</t>
         </is>
       </c>
-      <c r="D9" s="0" t="inlineStr">
+      <c r="D9" s="21" t="inlineStr">
         <is>
           <t>Needs a producer for OnsiteBoothContact AND an order-linkage (today keyed company_id+show_id, no Order FK).</t>
         </is>
       </c>
-      <c r="E9" s="0" t="inlineStr">
+      <c r="E9" s="21" t="inlineStr">
         <is>
           <t>SBE-1169 'View Onsite Boot Contact' + SBE-1171 'Edit On-Site Booth Contact'; producer/management SBE-1165 'Onsite Booth Contacts Management' (Epic SBE-1075 Exhibitor Onboarding).</t>
         </is>
       </c>
-      <c r="F9" s="0" t="inlineStr">
+      <c r="F9" s="21" t="inlineStr">
         <is>
           <t>SBE-1169/1171: Ritam Mondal; SBE-1165: Manish Gun</t>
         </is>
       </c>
-      <c r="G9" s="0" t="inlineStr">
+      <c r="G9" s="21" t="inlineStr">
         <is>
           <t>SBE-1169/1171: To Do, SBE Sprint 5. SBE-1165: To Do, backlog.</t>
         </is>
       </c>
-      <c r="H9" s="0" t="inlineStr">
+      <c r="H9" s="21" t="inlineStr">
         <is>
           <t>BLOCKED on SBE-1169 (+ SBE-1165). Confluence Edit story intends per-order onsite contact, so those stories add both the producer and the order-linkage.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="0" t="inlineStr">
+      <c r="A10" s="21" t="inlineStr">
         <is>
           <t>13.3-ac</t>
         </is>
       </c>
-      <c r="B10" s="0" t="inlineStr">
+      <c r="B10" s="21" t="inlineStr">
         <is>
           <t>Documents downloadable (invoice + agreement)</t>
         </is>
       </c>
-      <c r="C10" s="0" t="inlineStr">
+      <c r="C10" s="23" t="inlineStr">
         <is>
           <t>Blocked</t>
         </is>
       </c>
-      <c r="D10" s="0" t="inlineStr">
+      <c r="D10" s="21" t="inlineStr">
         <is>
           <t>Compound: invoice PDF downloadable AND signed agreement downloadable.</t>
         </is>
       </c>
-      <c r="E10" s="0" t="inlineStr">
+      <c r="E10" s="21" t="inlineStr">
         <is>
           <t>Invoice half -&gt; 13.3-s (Deferred, A-vs-B). Agreement half -&gt; 13.3-v (Blocked; Kshitiz SBE-862/869; reconcile SBE-1158).</t>
         </is>
       </c>
-      <c r="F10" s="0" t="inlineStr">
+      <c r="F10" s="21" t="inlineStr">
         <is>
           <t>see 13.3-s / 13.3-v</t>
         </is>
       </c>
-      <c r="G10" s="0" t="inlineStr">
+      <c r="G10" s="21" t="inlineStr">
         <is>
           <t>see 13.3-s / 13.3-v</t>
         </is>
       </c>
-      <c r="H10" s="0" t="inlineStr">
+      <c r="H10" s="21" t="inlineStr">
         <is>
           <t>BLOCKED. Tracked entirely via 13.3-s (invoice) and 13.3-v (agreement).</t>
         </is>
@@ -8083,168 +8125,168 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="0" t="inlineStr">
         <is>
           <t>Section</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="0" t="inlineStr">
         <is>
           <t>Detail</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="0" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="0" t="inlineStr">
         <is>
           <t>Not started — analysis/feasibility stage only. Verdicts revised 2026-07-01 (per-item review).</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="0" t="inlineStr">
         <is>
           <t>Branch</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="0" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="0" t="inlineStr">
         <is>
           <t>SBE ticket</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="0" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="0" t="inlineStr">
         <is>
           <t>Commits</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="0" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="0" t="inlineStr">
         <is>
           <t>PR</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="0" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="0" t="inlineStr">
         <is>
           <t>Swagger tag</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="0" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="0" t="inlineStr">
         <is>
           <t>Build gates (npm ci / prisma generate / typecheck / lint / test:cov / build)</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="0" t="inlineStr">
         <is>
           <t>— not run (unbuilt)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="0" t="inlineStr">
         <is>
           <t>Live smoke</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="0" t="inlineStr">
         <is>
           <t>— not run</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="0" t="inlineStr">
         <is>
           <t>Confirmed build scope (20 Deliverable)</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="0" t="inlineStr">
         <is>
           <t>GET /orders/:orderId aggregate — header (per-show shows[]), booth (size/price/subtotal), add-ons, sponsorships, financial summary, payment details, agreement acceptance, ownership scoping, reconciliation, per-item lines.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="0" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="0" t="inlineStr">
         <is>
           <t>Everything — nothing built yet.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="0" t="inlineStr">
         <is>
           <t>Not ready — see Open Questions register</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="0" t="inlineStr">
         <is>
           <t>6 Blocked (13.3-g, -l, -t, -v, -w, -ac) + 1 Deferred (13.3-s) + 2 Not Deliverable (13.3-c, -f). Full detail (question / blocking story + Jira / assignee / sprint / decision) is in the Open Questions sheet.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="0" t="inlineStr">
         <is>
           <t>External dependencies</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="0" t="inlineStr">
         <is>
           <t>See the Cross-Epic Dependencies sheet.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="0" t="inlineStr">
         <is>
           <t>Out of API scope</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="0" t="inlineStr">
         <is>
           <t>Front-end wiring (row-to-detail navigation, document download buttons) and anything marked Out of Scope.</t>
         </is>

</xml_diff>